<commit_message>
dump and search related issue fix
</commit_message>
<xml_diff>
--- a/sample/ReviewPackets_Sample.xlsx
+++ b/sample/ReviewPackets_Sample.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anurag Srivastava\Desktop\Learning\Practice\ReviewPacket\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDEBC4F8-E3C7-4BDD-A0C7-6E94BAEA9EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5A00F44-F685-48E5-85A5-F5966CF3BA40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="94">
   <si>
     <t>Issue Key</t>
   </si>
@@ -296,6 +296,12 @@
   </si>
   <si>
     <t>REL-2</t>
+  </si>
+  <si>
+    <t>abc</t>
+  </si>
+  <si>
+    <t>cdf</t>
   </si>
 </sst>
 </file>
@@ -331,8 +337,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -635,16 +644,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="27.21875" customWidth="1"/>
+    <col min="4" max="4" width="28.33203125" customWidth="1"/>
+    <col min="13" max="13" width="48.88671875" customWidth="1"/>
     <col min="15" max="15" width="26.21875" customWidth="1"/>
     <col min="17" max="17" width="16.109375" customWidth="1"/>
     <col min="18" max="18" width="14.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -696,8 +707,14 @@
       <c r="Q1" t="s">
         <v>1</v>
       </c>
+      <c r="R1" t="s">
+        <v>3</v>
+      </c>
+      <c r="S1" t="s">
+        <v>3</v>
+      </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -734,7 +751,7 @@
       <c r="L2" t="s">
         <v>26</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" s="1" t="s">
         <v>27</v>
       </c>
       <c r="P2" t="s">
@@ -743,8 +760,14 @@
       <c r="Q2" t="s">
         <v>29</v>
       </c>
+      <c r="R2" t="s">
+        <v>92</v>
+      </c>
+      <c r="S2" t="s">
+        <v>93</v>
+      </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -793,8 +816,14 @@
       <c r="P3" t="s">
         <v>40</v>
       </c>
+      <c r="R3">
+        <v>1</v>
+      </c>
+      <c r="S3">
+        <v>2</v>
+      </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>41</v>
       </c>
@@ -828,8 +857,14 @@
       <c r="L4" t="s">
         <v>47</v>
       </c>
+      <c r="R4">
+        <v>1</v>
+      </c>
+      <c r="S4">
+        <v>2</v>
+      </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>48</v>
       </c>
@@ -878,8 +913,14 @@
       <c r="Q5" t="s">
         <v>59</v>
       </c>
+      <c r="R5">
+        <v>1</v>
+      </c>
+      <c r="S5">
+        <v>2</v>
+      </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>60</v>
       </c>
@@ -922,8 +963,14 @@
       <c r="P6" t="s">
         <v>68</v>
       </c>
+      <c r="R6">
+        <v>1</v>
+      </c>
+      <c r="S6">
+        <v>2</v>
+      </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>69</v>
       </c>
@@ -975,8 +1022,14 @@
       <c r="Q7" t="s">
         <v>76</v>
       </c>
+      <c r="R7">
+        <v>1</v>
+      </c>
+      <c r="S7">
+        <v>2</v>
+      </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>77</v>
       </c>
@@ -1019,8 +1072,14 @@
       <c r="P8" t="s">
         <v>85</v>
       </c>
+      <c r="R8">
+        <v>1</v>
+      </c>
+      <c r="S8">
+        <v>2</v>
+      </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>86</v>
       </c>

</xml_diff>

<commit_message>
updated preview and review id extraction
</commit_message>
<xml_diff>
--- a/sample/ReviewPackets_Sample.xlsx
+++ b/sample/ReviewPackets_Sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anurag Srivastava\Desktop\Learning\Practice\ReviewPacket\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5A00F44-F685-48E5-85A5-F5966CF3BA40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB07DBFA-4036-47B0-90FD-0CB082DD068C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="124">
   <si>
     <t>Issue Key</t>
   </si>
@@ -302,6 +302,96 @@
   </si>
   <si>
     <t>cdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abcde 45467 </t>
+  </si>
+  <si>
+    <t>RP-111</t>
+  </si>
+  <si>
+    <t>RP-112</t>
+  </si>
+  <si>
+    <t>RP-113</t>
+  </si>
+  <si>
+    <t>RP-114</t>
+  </si>
+  <si>
+    <t>RP-115</t>
+  </si>
+  <si>
+    <t>RP-116</t>
+  </si>
+  <si>
+    <t>RP-117</t>
+  </si>
+  <si>
+    <t>RP-118</t>
+  </si>
+  <si>
+    <t>RP-121</t>
+  </si>
+  <si>
+    <t>RP-122</t>
+  </si>
+  <si>
+    <t>RP-123</t>
+  </si>
+  <si>
+    <t>RP-124</t>
+  </si>
+  <si>
+    <t>RP-125</t>
+  </si>
+  <si>
+    <t>RP-126</t>
+  </si>
+  <si>
+    <t>RP-127</t>
+  </si>
+  <si>
+    <t>RP-128</t>
+  </si>
+  <si>
+    <t>reviewid=46574</t>
+  </si>
+  <si>
+    <t>abc41443</t>
+  </si>
+  <si>
+    <t>review:id:22</t>
+  </si>
+  <si>
+    <t>review12312</t>
+  </si>
+  <si>
+    <t>id:31321</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abcde 45461 </t>
+  </si>
+  <si>
+    <t>reviewid:46572</t>
+  </si>
+  <si>
+    <t>ABFMS-46573</t>
+  </si>
+  <si>
+    <t>dqewdewfefewfreviewid:46534</t>
+  </si>
+  <si>
+    <t>fwfwfwfewfwe#reviewid:42574</t>
+  </si>
+  <si>
+    <t>fwfwfwfewfwe#review id = 16574</t>
+  </si>
+  <si>
+    <t>#46272</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abcde Review packet: 45417 </t>
   </si>
 </sst>
 </file>
@@ -337,11 +427,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -644,7 +735,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="27.21875" customWidth="1"/>
@@ -724,9 +815,6 @@
       <c r="C2" t="s">
         <v>18</v>
       </c>
-      <c r="D2" t="s">
-        <v>19</v>
-      </c>
       <c r="E2" t="s">
         <v>20</v>
       </c>
@@ -753,6 +841,9 @@
       </c>
       <c r="M2" s="1" t="s">
         <v>27</v>
+      </c>
+      <c r="O2" t="s">
+        <v>116</v>
       </c>
       <c r="P2" t="s">
         <v>28</v>
@@ -810,8 +901,8 @@
       <c r="N3" t="s">
         <v>39</v>
       </c>
-      <c r="O3">
-        <v>46574</v>
+      <c r="O3" t="s">
+        <v>117</v>
       </c>
       <c r="P3" t="s">
         <v>40</v>
@@ -857,6 +948,9 @@
       <c r="L4" t="s">
         <v>47</v>
       </c>
+      <c r="O4" t="s">
+        <v>118</v>
+      </c>
       <c r="R4">
         <v>1</v>
       </c>
@@ -907,6 +1001,9 @@
       <c r="N5" t="s">
         <v>57</v>
       </c>
+      <c r="O5" t="s">
+        <v>111</v>
+      </c>
       <c r="P5" t="s">
         <v>58</v>
       </c>
@@ -960,6 +1057,9 @@
       <c r="M6" t="s">
         <v>67</v>
       </c>
+      <c r="O6" t="s">
+        <v>119</v>
+      </c>
       <c r="P6" t="s">
         <v>68</v>
       </c>
@@ -1013,8 +1113,8 @@
       <c r="N7" t="s">
         <v>52</v>
       </c>
-      <c r="O7">
-        <v>46571</v>
+      <c r="O7" t="s">
+        <v>120</v>
       </c>
       <c r="P7" t="s">
         <v>75</v>
@@ -1069,6 +1169,12 @@
       <c r="M8" t="s">
         <v>84</v>
       </c>
+      <c r="N8" t="s">
+        <v>52</v>
+      </c>
+      <c r="O8" t="s">
+        <v>121</v>
+      </c>
       <c r="P8" t="s">
         <v>85</v>
       </c>
@@ -1122,10 +1228,864 @@
       <c r="N9" t="s">
         <v>52</v>
       </c>
-      <c r="O9">
+      <c r="O9" t="s">
+        <v>122</v>
+      </c>
+      <c r="P9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" t="s">
+        <v>22</v>
+      </c>
+      <c r="H10" t="s">
+        <v>23</v>
+      </c>
+      <c r="I10" t="s">
+        <v>24</v>
+      </c>
+      <c r="J10" t="s">
+        <v>25</v>
+      </c>
+      <c r="K10" t="s">
+        <v>19</v>
+      </c>
+      <c r="L10" t="s">
+        <v>26</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O10" t="s">
+        <v>123</v>
+      </c>
+      <c r="P10" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>29</v>
+      </c>
+      <c r="R10" t="s">
+        <v>92</v>
+      </c>
+      <c r="S10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11" t="s">
+        <v>22</v>
+      </c>
+      <c r="H11" t="s">
+        <v>35</v>
+      </c>
+      <c r="I11" t="s">
+        <v>36</v>
+      </c>
+      <c r="J11" t="s">
+        <v>37</v>
+      </c>
+      <c r="K11" t="s">
+        <v>32</v>
+      </c>
+      <c r="L11" t="s">
+        <v>26</v>
+      </c>
+      <c r="M11" t="s">
+        <v>38</v>
+      </c>
+      <c r="N11" t="s">
+        <v>39</v>
+      </c>
+      <c r="O11">
+        <v>3413413146574</v>
+      </c>
+      <c r="P11" t="s">
+        <v>40</v>
+      </c>
+      <c r="R11">
+        <v>1</v>
+      </c>
+      <c r="S11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>97</v>
+      </c>
+      <c r="B12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" t="s">
+        <v>21</v>
+      </c>
+      <c r="H12" t="s">
+        <v>44</v>
+      </c>
+      <c r="I12" t="s">
+        <v>45</v>
+      </c>
+      <c r="J12" t="s">
+        <v>46</v>
+      </c>
+      <c r="K12" t="s">
+        <v>43</v>
+      </c>
+      <c r="L12" t="s">
+        <v>47</v>
+      </c>
+      <c r="O12">
+        <v>13213</v>
+      </c>
+      <c r="R12">
+        <v>1</v>
+      </c>
+      <c r="S12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" t="s">
+        <v>51</v>
+      </c>
+      <c r="F13" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" t="s">
+        <v>53</v>
+      </c>
+      <c r="H13" t="s">
+        <v>54</v>
+      </c>
+      <c r="I13" t="s">
+        <v>55</v>
+      </c>
+      <c r="J13" t="s">
+        <v>25</v>
+      </c>
+      <c r="K13" t="s">
+        <v>50</v>
+      </c>
+      <c r="L13" t="s">
+        <v>47</v>
+      </c>
+      <c r="M13" t="s">
+        <v>56</v>
+      </c>
+      <c r="N13" t="s">
+        <v>57</v>
+      </c>
+      <c r="O13" t="s">
+        <v>112</v>
+      </c>
+      <c r="P13" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>59</v>
+      </c>
+      <c r="R13">
+        <v>1</v>
+      </c>
+      <c r="S13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>99</v>
+      </c>
+      <c r="B14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D14" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" t="s">
+        <v>63</v>
+      </c>
+      <c r="H14" t="s">
+        <v>64</v>
+      </c>
+      <c r="I14" t="s">
+        <v>65</v>
+      </c>
+      <c r="J14" t="s">
+        <v>46</v>
+      </c>
+      <c r="K14" t="s">
+        <v>50</v>
+      </c>
+      <c r="L14" t="s">
+        <v>66</v>
+      </c>
+      <c r="M14" t="s">
+        <v>67</v>
+      </c>
+      <c r="O14">
+        <v>41241</v>
+      </c>
+      <c r="P14" t="s">
+        <v>68</v>
+      </c>
+      <c r="R14">
+        <v>1</v>
+      </c>
+      <c r="S14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>100</v>
+      </c>
+      <c r="B15" t="s">
+        <v>70</v>
+      </c>
+      <c r="C15" t="s">
+        <v>62</v>
+      </c>
+      <c r="D15" t="s">
+        <v>71</v>
+      </c>
+      <c r="E15" t="s">
+        <v>33</v>
+      </c>
+      <c r="F15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" t="s">
+        <v>62</v>
+      </c>
+      <c r="H15" t="s">
+        <v>72</v>
+      </c>
+      <c r="I15" t="s">
+        <v>73</v>
+      </c>
+      <c r="J15" t="s">
+        <v>25</v>
+      </c>
+      <c r="K15" t="s">
+        <v>71</v>
+      </c>
+      <c r="L15" t="s">
+        <v>66</v>
+      </c>
+      <c r="M15" t="s">
+        <v>74</v>
+      </c>
+      <c r="N15" t="s">
+        <v>52</v>
+      </c>
+      <c r="O15">
+        <v>46371</v>
+      </c>
+      <c r="P15" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>76</v>
+      </c>
+      <c r="R15">
+        <v>1</v>
+      </c>
+      <c r="S15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>101</v>
+      </c>
+      <c r="B16" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16" t="s">
+        <v>33</v>
+      </c>
+      <c r="F16" t="s">
+        <v>79</v>
+      </c>
+      <c r="G16" t="s">
+        <v>80</v>
+      </c>
+      <c r="H16" t="s">
+        <v>81</v>
+      </c>
+      <c r="I16" t="s">
+        <v>82</v>
+      </c>
+      <c r="J16" t="s">
+        <v>25</v>
+      </c>
+      <c r="K16" t="s">
+        <v>43</v>
+      </c>
+      <c r="L16" t="s">
+        <v>83</v>
+      </c>
+      <c r="M16" t="s">
+        <v>84</v>
+      </c>
+      <c r="O16" t="s">
+        <v>113</v>
+      </c>
+      <c r="P16" t="s">
+        <v>85</v>
+      </c>
+      <c r="R16">
+        <v>1</v>
+      </c>
+      <c r="S16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" t="s">
+        <v>87</v>
+      </c>
+      <c r="C17" t="s">
+        <v>80</v>
+      </c>
+      <c r="D17" t="s">
+        <v>32</v>
+      </c>
+      <c r="E17" t="s">
+        <v>51</v>
+      </c>
+      <c r="F17" t="s">
+        <v>52</v>
+      </c>
+      <c r="G17" t="s">
+        <v>88</v>
+      </c>
+      <c r="H17" t="s">
+        <v>54</v>
+      </c>
+      <c r="I17" t="s">
+        <v>89</v>
+      </c>
+      <c r="J17" t="s">
+        <v>46</v>
+      </c>
+      <c r="K17" t="s">
+        <v>32</v>
+      </c>
+      <c r="L17" t="s">
+        <v>83</v>
+      </c>
+      <c r="M17" t="s">
+        <v>90</v>
+      </c>
+      <c r="N17" t="s">
+        <v>52</v>
+      </c>
+      <c r="O17">
         <v>46572</v>
       </c>
-      <c r="P9" t="s">
+      <c r="P17" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="E18" t="s">
+        <v>20</v>
+      </c>
+      <c r="F18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" t="s">
+        <v>22</v>
+      </c>
+      <c r="H18" t="s">
+        <v>23</v>
+      </c>
+      <c r="I18" t="s">
+        <v>24</v>
+      </c>
+      <c r="J18" t="s">
+        <v>25</v>
+      </c>
+      <c r="K18" t="s">
+        <v>19</v>
+      </c>
+      <c r="L18" t="s">
+        <v>26</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O18" t="s">
+        <v>94</v>
+      </c>
+      <c r="P18" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>29</v>
+      </c>
+      <c r="R18" t="s">
+        <v>92</v>
+      </c>
+      <c r="S18" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>104</v>
+      </c>
+      <c r="B19" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" t="s">
+        <v>32</v>
+      </c>
+      <c r="E19" t="s">
+        <v>33</v>
+      </c>
+      <c r="F19" t="s">
+        <v>34</v>
+      </c>
+      <c r="G19" t="s">
+        <v>22</v>
+      </c>
+      <c r="H19" t="s">
+        <v>35</v>
+      </c>
+      <c r="I19" t="s">
+        <v>36</v>
+      </c>
+      <c r="J19" t="s">
+        <v>37</v>
+      </c>
+      <c r="K19" t="s">
+        <v>32</v>
+      </c>
+      <c r="L19" t="s">
+        <v>26</v>
+      </c>
+      <c r="M19" t="s">
+        <v>38</v>
+      </c>
+      <c r="N19" t="s">
+        <v>39</v>
+      </c>
+      <c r="O19">
+        <v>46574</v>
+      </c>
+      <c r="P19" t="s">
+        <v>40</v>
+      </c>
+      <c r="R19">
+        <v>1</v>
+      </c>
+      <c r="S19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>105</v>
+      </c>
+      <c r="B20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" t="s">
+        <v>43</v>
+      </c>
+      <c r="E20" t="s">
+        <v>20</v>
+      </c>
+      <c r="F20" t="s">
+        <v>21</v>
+      </c>
+      <c r="H20" t="s">
+        <v>44</v>
+      </c>
+      <c r="I20" t="s">
+        <v>45</v>
+      </c>
+      <c r="J20" t="s">
+        <v>46</v>
+      </c>
+      <c r="K20" t="s">
+        <v>43</v>
+      </c>
+      <c r="L20" t="s">
+        <v>47</v>
+      </c>
+      <c r="O20" s="2">
+        <v>230000000000000</v>
+      </c>
+      <c r="R20">
+        <v>1</v>
+      </c>
+      <c r="S20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>106</v>
+      </c>
+      <c r="B21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" t="s">
+        <v>22</v>
+      </c>
+      <c r="D21" t="s">
+        <v>50</v>
+      </c>
+      <c r="E21" t="s">
+        <v>51</v>
+      </c>
+      <c r="F21" t="s">
+        <v>52</v>
+      </c>
+      <c r="G21" t="s">
+        <v>53</v>
+      </c>
+      <c r="H21" t="s">
+        <v>54</v>
+      </c>
+      <c r="I21" t="s">
+        <v>55</v>
+      </c>
+      <c r="J21" t="s">
+        <v>25</v>
+      </c>
+      <c r="K21" t="s">
+        <v>50</v>
+      </c>
+      <c r="L21" t="s">
+        <v>47</v>
+      </c>
+      <c r="M21" t="s">
+        <v>56</v>
+      </c>
+      <c r="N21" t="s">
+        <v>57</v>
+      </c>
+      <c r="O21" t="s">
+        <v>114</v>
+      </c>
+      <c r="P21" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>59</v>
+      </c>
+      <c r="R21">
+        <v>1</v>
+      </c>
+      <c r="S21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>107</v>
+      </c>
+      <c r="B22" t="s">
+        <v>61</v>
+      </c>
+      <c r="C22" t="s">
+        <v>62</v>
+      </c>
+      <c r="D22" t="s">
+        <v>50</v>
+      </c>
+      <c r="E22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F22" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" t="s">
+        <v>63</v>
+      </c>
+      <c r="H22" t="s">
+        <v>64</v>
+      </c>
+      <c r="I22" t="s">
+        <v>65</v>
+      </c>
+      <c r="J22" t="s">
+        <v>46</v>
+      </c>
+      <c r="K22" t="s">
+        <v>50</v>
+      </c>
+      <c r="L22" t="s">
+        <v>66</v>
+      </c>
+      <c r="M22" t="s">
+        <v>67</v>
+      </c>
+      <c r="O22" t="s">
+        <v>115</v>
+      </c>
+      <c r="P22" t="s">
+        <v>68</v>
+      </c>
+      <c r="R22">
+        <v>1</v>
+      </c>
+      <c r="S22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>108</v>
+      </c>
+      <c r="B23" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" t="s">
+        <v>62</v>
+      </c>
+      <c r="D23" t="s">
+        <v>71</v>
+      </c>
+      <c r="E23" t="s">
+        <v>33</v>
+      </c>
+      <c r="F23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" t="s">
+        <v>62</v>
+      </c>
+      <c r="H23" t="s">
+        <v>72</v>
+      </c>
+      <c r="I23" t="s">
+        <v>73</v>
+      </c>
+      <c r="J23" t="s">
+        <v>25</v>
+      </c>
+      <c r="K23" t="s">
+        <v>71</v>
+      </c>
+      <c r="L23" t="s">
+        <v>66</v>
+      </c>
+      <c r="M23" t="s">
+        <v>74</v>
+      </c>
+      <c r="N23" t="s">
+        <v>52</v>
+      </c>
+      <c r="O23">
+        <v>46371</v>
+      </c>
+      <c r="P23" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>76</v>
+      </c>
+      <c r="R23">
+        <v>1</v>
+      </c>
+      <c r="S23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>109</v>
+      </c>
+      <c r="B24" t="s">
+        <v>78</v>
+      </c>
+      <c r="C24" t="s">
+        <v>63</v>
+      </c>
+      <c r="D24" t="s">
+        <v>43</v>
+      </c>
+      <c r="E24" t="s">
+        <v>33</v>
+      </c>
+      <c r="F24" t="s">
+        <v>79</v>
+      </c>
+      <c r="G24" t="s">
+        <v>80</v>
+      </c>
+      <c r="H24" t="s">
+        <v>81</v>
+      </c>
+      <c r="I24" t="s">
+        <v>82</v>
+      </c>
+      <c r="J24" t="s">
+        <v>25</v>
+      </c>
+      <c r="K24" t="s">
+        <v>43</v>
+      </c>
+      <c r="L24" t="s">
+        <v>83</v>
+      </c>
+      <c r="M24" t="s">
+        <v>84</v>
+      </c>
+      <c r="O24">
+        <v>41414</v>
+      </c>
+      <c r="P24" t="s">
+        <v>85</v>
+      </c>
+      <c r="R24">
+        <v>1</v>
+      </c>
+      <c r="S24">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>110</v>
+      </c>
+      <c r="B25" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" t="s">
+        <v>80</v>
+      </c>
+      <c r="D25" t="s">
+        <v>32</v>
+      </c>
+      <c r="E25" t="s">
+        <v>51</v>
+      </c>
+      <c r="F25" t="s">
+        <v>52</v>
+      </c>
+      <c r="G25" t="s">
+        <v>88</v>
+      </c>
+      <c r="H25" t="s">
+        <v>54</v>
+      </c>
+      <c r="I25" t="s">
+        <v>89</v>
+      </c>
+      <c r="J25" t="s">
+        <v>46</v>
+      </c>
+      <c r="K25" t="s">
+        <v>32</v>
+      </c>
+      <c r="L25" t="s">
+        <v>83</v>
+      </c>
+      <c r="M25" t="s">
+        <v>90</v>
+      </c>
+      <c r="N25" t="s">
+        <v>52</v>
+      </c>
+      <c r="O25">
+        <v>42272</v>
+      </c>
+      <c r="P25" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added collaborator preview word size
</commit_message>
<xml_diff>
--- a/sample/ReviewPackets_Sample.xlsx
+++ b/sample/ReviewPackets_Sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anurag Srivastava\Desktop\Learning\Practice\ReviewPacket\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB07DBFA-4036-47B0-90FD-0CB082DD068C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5014A5F2-0C47-4E21-801A-9FC578FBD0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="125">
   <si>
     <t>Issue Key</t>
   </si>
@@ -392,6 +392,44 @@
   </si>
   <si>
     <t xml:space="preserve">abcde Review packet: 45417 </t>
+  </si>
+  <si>
+    <t>Must accept terms
+Must accept terms 
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms 
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms 
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms 
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms 
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms 
+Must accept terms
+Must accept terms
+Must accept terms
+Must accept terms</t>
   </si>
 </sst>
 </file>
@@ -805,7 +843,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -840,7 +878,7 @@
         <v>26</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>27</v>
+        <v>124</v>
       </c>
       <c r="O2" t="s">
         <v>116</v>
@@ -1447,7 +1485,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:19" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>99</v>
       </c>
@@ -1484,8 +1522,8 @@
       <c r="L14" t="s">
         <v>66</v>
       </c>
-      <c r="M14" t="s">
-        <v>67</v>
+      <c r="M14" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="O14">
         <v>41241</v>
@@ -1612,7 +1650,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:19" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>102</v>
       </c>
@@ -1649,8 +1687,8 @@
       <c r="L17" t="s">
         <v>83</v>
       </c>
-      <c r="M17" t="s">
-        <v>90</v>
+      <c r="M17" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="N17" t="s">
         <v>52</v>

</xml_diff>

<commit_message>
Added missing custom fields and updated url to aero
</commit_message>
<xml_diff>
--- a/sample/ReviewPackets_Sample.xlsx
+++ b/sample/ReviewPackets_Sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anurag Srivastava\Desktop\Learning\Practice\ReviewPacket\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5014A5F2-0C47-4E21-801A-9FC578FBD0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC841354-8D44-4745-9BA2-A7C09F0D8EB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="132">
   <si>
     <t>Issue Key</t>
   </si>
@@ -430,6 +430,27 @@
 Must accept terms
 Must accept terms
 Must accept terms</t>
+  </si>
+  <si>
+    <t>Custom field (Category of Task)</t>
+  </si>
+  <si>
+    <t>Custom field (Affected Subsystem/s)</t>
+  </si>
+  <si>
+    <t>Custom field (Epic Link)</t>
+  </si>
+  <si>
+    <t>Custom field (Acceptance Criteria)</t>
+  </si>
+  <si>
+    <t>Custom field (Solution)</t>
+  </si>
+  <si>
+    <t>Custom field (Review Info)</t>
+  </si>
+  <si>
+    <t>Custom field (Issue Links)</t>
   </si>
 </sst>
 </file>
@@ -773,7 +794,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S25"/>
+  <dimension ref="A1:AM25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="27.21875" customWidth="1"/>
@@ -784,7 +805,7 @@
     <col min="18" max="18" width="14.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -842,8 +863,29 @@
       <c r="S1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:19" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="U1" t="s">
+        <v>125</v>
+      </c>
+      <c r="X1" t="s">
+        <v>126</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>127</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>128</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>129</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>130</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:39" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -896,7 +938,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -952,7 +994,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>41</v>
       </c>
@@ -996,7 +1038,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>48</v>
       </c>
@@ -1055,7 +1097,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>60</v>
       </c>
@@ -1108,7 +1150,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>69</v>
       </c>
@@ -1167,7 +1209,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>77</v>
       </c>
@@ -1223,7 +1265,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>86</v>
       </c>
@@ -1273,7 +1315,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>95</v>
       </c>
@@ -1326,7 +1368,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1382,7 +1424,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>97</v>
       </c>
@@ -1426,7 +1468,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>98</v>
       </c>
@@ -1485,7 +1527,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:39" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>99</v>
       </c>
@@ -1538,7 +1580,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>100</v>
       </c>
@@ -1597,7 +1639,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>101</v>
       </c>

</xml_diff>